<commit_message>
new retrieval sequence files that dont have regularities in left right responses anymore
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_01.xlsx
+++ b/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_01.xlsx
@@ -609,12 +609,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P2" t="n">
@@ -802,17 +802,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P4" t="n">
@@ -823,7 +823,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S4" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S5" t="n">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P6" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S6" t="n">
@@ -1104,12 +1104,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P7" t="n">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1188,22 +1188,22 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S8" t="n">
@@ -1232,10 +1232,10 @@
         <v>1</v>
       </c>
       <c r="V8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="W8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1302,12 +1302,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P9" t="n">
@@ -1366,12 +1366,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1410,10 +1410,10 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.4</v>
+        <v>0.47</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1430,10 +1430,10 @@
         <v>2</v>
       </c>
       <c r="V10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1512,7 +1512,7 @@
         <v>0.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
         <v>13</v>
       </c>
       <c r="W11" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1599,19 +1599,19 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P12" t="n">
         <v>0.73</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
         <v>12</v>
       </c>
       <c r="W12" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1703,18 +1703,18 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P13" t="n">
         <v>0.67</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.27</v>
+        <v>0.47</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S13" t="n">
@@ -1730,7 +1730,7 @@
         <v>7</v>
       </c>
       <c r="W13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1787,33 +1787,33 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P14" t="n">
         <v>0.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.47</v>
+        <v>0.27</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S14" t="n">
@@ -1829,7 +1829,7 @@
         <v>13</v>
       </c>
       <c r="W14" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1896,19 +1896,19 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P15" t="n">
         <v>0.75</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -1928,7 +1928,7 @@
         <v>6</v>
       </c>
       <c r="W15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1995,19 +1995,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P16" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         <v>3</v>
       </c>
       <c r="W16" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2084,17 +2084,17 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2106,11 +2106,11 @@
         <v>0.8</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.58</v>
+        <v>0.31</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S17" t="n">
@@ -2126,7 +2126,7 @@
         <v>10</v>
       </c>
       <c r="W17" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2188,28 +2188,28 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.42</v>
+        <v>0.64</v>
       </c>
       <c r="Q18" t="n">
         <v>0.2</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S18" t="n">
@@ -2222,7 +2222,7 @@
         <v>10</v>
       </c>
       <c r="V18" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="W18" t="n">
         <v>13</v>
@@ -2287,17 +2287,17 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P19" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S19" t="n">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2386,12 +2386,12 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2400,14 +2400,14 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="Q20" t="n">
         <v>0.4</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S20" t="n">
@@ -2420,7 +2420,7 @@
         <v>8</v>
       </c>
       <c r="V20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W20" t="n">
         <v>12</v>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2480,33 +2480,33 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P21" t="n">
         <v>0.75</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S21" t="n">
@@ -2522,7 +2522,7 @@
         <v>2</v>
       </c>
       <c r="W21" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -2554,12 +2554,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2574,38 +2574,38 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>0.75</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.64</v>
+        <v>0.58</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S22" t="n">
@@ -2618,10 +2618,10 @@
         <v>5</v>
       </c>
       <c r="V22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="W22" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2693,18 +2693,18 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.64</v>
+        <v>0.33</v>
       </c>
       <c r="Q23" t="n">
         <v>0.2</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S23" t="n">
@@ -2717,7 +2717,7 @@
         <v>2</v>
       </c>
       <c r="V23" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="W23" t="n">
         <v>8</v>
@@ -2752,12 +2752,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2787,19 +2787,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.4</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.2</v>
+        <v>0.47</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -2816,10 +2816,10 @@
         <v>4</v>
       </c>
       <c r="V24" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="W24" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -2851,12 +2851,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2871,17 +2871,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2891,18 +2891,18 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.53</v>
+        <v>0.27</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S25" t="n">
@@ -2915,10 +2915,10 @@
         <v>9</v>
       </c>
       <c r="V25" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="W25" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2970,22 +2970,22 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2994,14 +2994,14 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.73</v>
+        <v>0.53</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S26" t="n">
@@ -3014,10 +3014,10 @@
         <v>14</v>
       </c>
       <c r="V26" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="W26" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3084,16 +3084,16 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.53</v>
+        <v>0.67</v>
       </c>
       <c r="Q27" t="n">
         <v>0.27</v>
@@ -3113,7 +3113,7 @@
         <v>16</v>
       </c>
       <c r="V27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W27" t="n">
         <v>2</v>
@@ -3148,12 +3148,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3168,38 +3168,38 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S28" t="n">
@@ -3212,10 +3212,10 @@
         <v>13</v>
       </c>
       <c r="V28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W28" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29">
@@ -3247,12 +3247,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3267,17 +3267,17 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3287,18 +3287,18 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>0.53</v>
+        <v>0.64</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S29" t="n">
@@ -3311,10 +3311,10 @@
         <v>7</v>
       </c>
       <c r="V29" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W29" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30">
@@ -3346,12 +3346,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3366,12 +3366,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3390,10 +3390,10 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.58</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -3410,10 +3410,10 @@
         <v>6</v>
       </c>
       <c r="V30" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W30" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
@@ -3445,14 +3445,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>flower</t>
@@ -3465,38 +3465,38 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>chair</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>lamp</t>
-        </is>
-      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P31" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q31" t="n">
         <v>0.53</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0.42</v>
-      </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S31" t="n">
@@ -3509,10 +3509,10 @@
         <v>10</v>
       </c>
       <c r="V31" t="n">
+        <v>3</v>
+      </c>
+      <c r="W31" t="n">
         <v>4</v>
-      </c>
-      <c r="W31" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="32">
@@ -3544,12 +3544,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3564,12 +3564,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3588,10 +3588,10 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.58</v>
+        <v>0.47</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -3608,10 +3608,10 @@
         <v>3</v>
       </c>
       <c r="V32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W32" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33">
@@ -3678,12 +3678,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P33" t="n">
@@ -3772,17 +3772,17 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P34" t="n">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S34" t="n">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3881,18 +3881,18 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="Q35" t="n">
         <v>0.2</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S35" t="n">
@@ -3905,7 +3905,7 @@
         <v>5</v>
       </c>
       <c r="V35" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="W35" t="n">
         <v>3</v>
@@ -3940,12 +3940,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3960,12 +3960,12 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3975,19 +3975,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -4004,10 +4004,10 @@
         <v>2</v>
       </c>
       <c r="V36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="W36" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4059,12 +4059,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4074,19 +4074,19 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.75</v>
+        <v>0.53</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.53</v>
+        <v>0.2</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>4</v>
       </c>
       <c r="V37" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="W37" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4138,12 +4138,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4158,38 +4158,38 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S38" t="n">
@@ -4202,10 +4202,10 @@
         <v>9</v>
       </c>
       <c r="V38" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="W38" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/guitar/guitar_19.jpg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4257,12 +4257,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4272,19 +4272,19 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -4301,10 +4301,10 @@
         <v>14</v>
       </c>
       <c r="V39" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="W39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -4336,12 +4336,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4356,22 +4356,22 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -4380,14 +4380,14 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S40" t="n">
@@ -4400,10 +4400,10 @@
         <v>16</v>
       </c>
       <c r="V40" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="W40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -4435,12 +4435,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4455,12 +4455,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4470,19 +4470,19 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.8</v>
+        <v>0.53</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.42</v>
+        <v>0.2</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -4499,10 +4499,10 @@
         <v>13</v>
       </c>
       <c r="V41" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="W41" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42">
@@ -4534,12 +4534,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4554,38 +4554,38 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.58</v>
+        <v>0.47</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.42</v>
+        <v>0.31</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S42" t="n">
@@ -4598,10 +4598,10 @@
         <v>7</v>
       </c>
       <c r="V42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W42" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.75</v>
       </c>
       <c r="Q43" t="n">
         <v>0.42</v>
@@ -4697,7 +4697,7 @@
         <v>6</v>
       </c>
       <c r="V43" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="W43" t="n">
         <v>9</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4757,33 +4757,33 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P44" t="n">
         <v>0.64</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.53</v>
+        <v>0.36</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S44" t="n">
@@ -4799,7 +4799,7 @@
         <v>5</v>
       </c>
       <c r="W44" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4856,12 +4856,12 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -4871,18 +4871,18 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P45" t="n">
         <v>0.8</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.47</v>
+        <v>0.58</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S45" t="n">
@@ -4898,7 +4898,7 @@
         <v>8</v>
       </c>
       <c r="W45" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
@@ -4930,12 +4930,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4950,38 +4950,38 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.47</v>
+        <v>0.27</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S46" t="n">
@@ -4994,10 +4994,10 @@
         <v>8</v>
       </c>
       <c r="V46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W46" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47">
@@ -5059,17 +5059,17 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P47" t="n">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S47" t="n">
@@ -5163,12 +5163,12 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P48" t="n">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5252,17 +5252,17 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -5274,11 +5274,11 @@
         <v>0.6</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S49" t="n">
@@ -5294,7 +5294,7 @@
         <v>12</v>
       </c>
       <c r="W49" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -5326,12 +5326,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5346,12 +5346,12 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -5370,10 +5370,10 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.33</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -5390,10 +5390,10 @@
         <v>4</v>
       </c>
       <c r="V50" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="W50" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51">
@@ -5425,12 +5425,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/fish/fish_03.jpg</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5445,38 +5445,38 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>fish</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.53</v>
+        <v>0.4</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S51" t="n">
@@ -5489,10 +5489,10 @@
         <v>9</v>
       </c>
       <c r="V51" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="W51" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -5559,12 +5559,12 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P52" t="n">
@@ -5623,12 +5623,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/guitar/guitar_19.jpg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5643,12 +5643,12 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -5658,19 +5658,19 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>0.47</v>
+        <v>0.8</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -5687,10 +5687,10 @@
         <v>16</v>
       </c>
       <c r="V53" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="W53" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -5757,16 +5757,16 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>0.8</v>
+        <v>0.64</v>
       </c>
       <c r="Q54" t="n">
         <v>0.31</v>
@@ -5786,7 +5786,7 @@
         <v>13</v>
       </c>
       <c r="V54" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W54" t="n">
         <v>9</v>
@@ -5821,12 +5821,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -5856,19 +5856,19 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.53</v>
+        <v>0.75</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.31</v>
+        <v>0.25</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -5885,10 +5885,10 @@
         <v>7</v>
       </c>
       <c r="V55" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W55" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56">
@@ -5920,12 +5920,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5940,38 +5940,38 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P56" t="n">
-        <v>0.47</v>
+        <v>0.58</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.31</v>
+        <v>0.42</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S56" t="n">
@@ -5984,10 +5984,10 @@
         <v>6</v>
       </c>
       <c r="V56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W56" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57">
@@ -6019,12 +6019,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6039,17 +6039,17 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -6059,18 +6059,18 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.53</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.58</v>
+        <v>0.36</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S57" t="n">
@@ -6083,10 +6083,10 @@
         <v>10</v>
       </c>
       <c r="V57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W57" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6143,33 +6143,33 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P58" t="n">
         <v>0.8</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.47</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S58" t="n">
@@ -6185,7 +6185,7 @@
         <v>8</v>
       </c>
       <c r="W58" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6237,12 +6237,12 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -6252,19 +6252,19 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>0.33</v>
+        <v>0.8</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.2</v>
+        <v>0.58</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
@@ -6281,10 +6281,10 @@
         <v>8</v>
       </c>
       <c r="V59" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="W59" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P60" t="n">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S60" t="n">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>stimuli/fish/fish_03.jpg</t>
+          <t>stimuli/guitar/guitar_19.jpg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6440,33 +6440,33 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>fish</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P61" t="n">
         <v>0.75</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.53</v>
+        <v>0.47</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S61" t="n">
@@ -6482,7 +6482,7 @@
         <v>4</v>
       </c>
       <c r="W61" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62">
@@ -6514,14 +6514,14 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
+          <t>stimuli/pencil/pencil_27.jpg</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
           <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>stimuli/bread/bread_21.jpg</t>
-        </is>
-      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>dog</t>
@@ -6534,38 +6534,38 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
           <t>flower</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>bread</t>
-        </is>
-      </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P62" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="Q62" t="n">
         <v>0.4</v>
       </c>
-      <c r="Q62" t="n">
-        <v>0.27</v>
-      </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S62" t="n">
@@ -6578,10 +6578,10 @@
         <v>2</v>
       </c>
       <c r="V62" t="n">
+        <v>16</v>
+      </c>
+      <c r="W62" t="n">
         <v>6</v>
-      </c>
-      <c r="W62" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="63">
@@ -6613,14 +6613,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
+          <t>stimuli/fish/fish_03.jpg</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
           <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>stimuli/ball/ball_31.jpg</t>
-        </is>
-      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>bicycle</t>
@@ -6633,22 +6633,22 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
           <t>hammer</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>ball</t>
-        </is>
-      </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -6657,14 +6657,14 @@
         </is>
       </c>
       <c r="P63" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="Q63" t="n">
         <v>0.53</v>
       </c>
-      <c r="Q63" t="n">
-        <v>0.2</v>
-      </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S63" t="n">
@@ -6677,10 +6677,10 @@
         <v>4</v>
       </c>
       <c r="V63" t="n">
+        <v>12</v>
+      </c>
+      <c r="W63" t="n">
         <v>7</v>
-      </c>
-      <c r="W63" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -6712,12 +6712,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>stimuli/fish/fish_03.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6732,12 +6732,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>fish</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -6747,19 +6747,19 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P64" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
@@ -6776,10 +6776,10 @@
         <v>9</v>
       </c>
       <c r="V64" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="W64" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -6811,12 +6811,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6831,22 +6831,22 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -6855,14 +6855,14 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>0.53</v>
+        <v>0.6</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S65" t="n">
@@ -6875,10 +6875,10 @@
         <v>14</v>
       </c>
       <c r="V65" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="W65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -6910,12 +6910,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/fish/fish_03.jpg</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6930,22 +6930,22 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>guitar</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>fish</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -6954,14 +6954,14 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>0.8</v>
+        <v>0.53</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S66" t="n">
@@ -6974,10 +6974,10 @@
         <v>16</v>
       </c>
       <c r="V66" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="W66" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -7029,7 +7029,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -7039,28 +7039,28 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="Q67" t="n">
         <v>0.31</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S67" t="n">
@@ -7073,7 +7073,7 @@
         <v>13</v>
       </c>
       <c r="V67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W67" t="n">
         <v>9</v>
@@ -7108,12 +7108,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7128,38 +7128,38 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P68" t="n">
-        <v>0.58</v>
+        <v>0.75</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.25</v>
+        <v>0.53</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S68" t="n">
@@ -7172,10 +7172,10 @@
         <v>7</v>
       </c>
       <c r="V68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="W68" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
+          <t>stimuli/pencil/pencil_27.jpg</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7232,17 +7232,17 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>lamp</t>
+          <t>pencil</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -7254,11 +7254,11 @@
         <v>0.58</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S69" t="n">
@@ -7274,7 +7274,7 @@
         <v>5</v>
       </c>
       <c r="W69" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="70">
@@ -7306,12 +7306,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7326,38 +7326,38 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P70" t="n">
-        <v>0.75</v>
+        <v>0.53</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S70" t="n">
@@ -7370,10 +7370,10 @@
         <v>10</v>
       </c>
       <c r="V70" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W70" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="71">
@@ -7435,17 +7435,17 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P71" t="n">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S71" t="n">
@@ -7504,12 +7504,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7524,38 +7524,38 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>0.8</v>
+        <v>0.53</v>
       </c>
       <c r="Q72" t="n">
-        <v>0.64</v>
+        <v>0.27</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S72" t="n">
@@ -7568,10 +7568,10 @@
         <v>8</v>
       </c>
       <c r="V72" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="W72" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
@@ -7603,7 +7603,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/guitar/guitar_19.jpg</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -7643,18 +7643,18 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>0.53</v>
+        <v>0.4</v>
       </c>
       <c r="Q73" t="n">
         <v>0.2</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S73" t="n">
@@ -7667,7 +7667,7 @@
         <v>1</v>
       </c>
       <c r="V73" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="W73" t="n">
         <v>10</v>
@@ -7702,7 +7702,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/lamp/lamp_18.jpg</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -7732,28 +7732,28 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P74" t="n">
-        <v>0.4</v>
+        <v>0.64</v>
       </c>
       <c r="Q74" t="n">
         <v>0.2</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S74" t="n">
@@ -7766,7 +7766,7 @@
         <v>5</v>
       </c>
       <c r="V74" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="W74" t="n">
         <v>3</v>
@@ -7836,12 +7836,12 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P75" t="n">
@@ -7900,12 +7900,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7920,38 +7920,38 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>pencil</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="P76" t="n">
-        <v>0.8</v>
+        <v>0.47</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.27</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="S76" t="n">
@@ -7964,10 +7964,10 @@
         <v>4</v>
       </c>
       <c r="V76" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="W76" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -8029,12 +8029,12 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>right</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -8050,7 +8050,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S77" t="n">
@@ -8098,14 +8098,14 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
+          <t>stimuli/pencil/pencil_27.jpg</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
           <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_47.jpg</t>
-        </is>
-      </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>house</t>
@@ -8118,38 +8118,38 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
           <t>hammer</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>hand</t>
-        </is>
-      </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>center</t>
         </is>
       </c>
       <c r="P78" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q78" t="n">
         <v>0.67</v>
       </c>
-      <c r="Q78" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="S78" t="n">
@@ -8162,10 +8162,10 @@
         <v>14</v>
       </c>
       <c r="V78" t="n">
+        <v>16</v>
+      </c>
+      <c r="W78" t="n">
         <v>7</v>
-      </c>
-      <c r="W78" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="79">
@@ -8197,12 +8197,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/guitar/guitar_19.jpg</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>stimuli/fish/fish_03.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8217,17 +8217,17 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>guitar</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>fish</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -8237,18 +8237,18 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="P79" t="n">
-        <v>0.53</v>
+        <v>0.8</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="S79" t="n">
@@ -8261,10 +8261,10 @@
         <v>16</v>
       </c>
       <c r="V79" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="W79" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new condition files for old localizer version and updated main task practice trial image
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_01.xlsx
+++ b/psychopy_exp_files/sequences/learning_block1_fixed-middle-10_01.xlsx
@@ -574,12 +574,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -594,12 +594,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -638,10 +638,10 @@
         <v>13</v>
       </c>
       <c r="V2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -668,19 +668,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>stimuli/flower/flower_32.jpg</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>guitar</t>
@@ -688,17 +688,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>hammer</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>jacket</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>bicycle</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -734,13 +734,13 @@
         <v>13</v>
       </c>
       <c r="U3" t="n">
+        <v>6</v>
+      </c>
+      <c r="V3" t="n">
+        <v>3</v>
+      </c>
+      <c r="W3" t="n">
         <v>7</v>
-      </c>
-      <c r="V3" t="n">
-        <v>10</v>
-      </c>
-      <c r="W3" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -762,42 +762,42 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -830,16 +830,16 @@
         <v>4</v>
       </c>
       <c r="T4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="W4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -861,42 +861,42 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>stimuli/hand/hand_47.jpg</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>stimuli/bread/bread_21.jpg</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>stimuli/dog/dog_21.jpg</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>hand</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>jacket</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>bread</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>dog</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -929,16 +929,16 @@
         <v>5</v>
       </c>
       <c r="T5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
+        <v>3</v>
+      </c>
+      <c r="V5" t="n">
+        <v>8</v>
+      </c>
+      <c r="W5" t="n">
         <v>10</v>
-      </c>
-      <c r="V5" t="n">
-        <v>3</v>
-      </c>
-      <c r="W5" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -960,17 +960,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -980,17 +980,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1028,13 +1028,13 @@
         <v>6</v>
       </c>
       <c r="T6" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W6" t="n">
         <v>14</v>
@@ -1059,17 +1059,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1079,17 +1079,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1127,13 +1127,13 @@
         <v>7</v>
       </c>
       <c r="T7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V7" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W7" t="n">
         <v>16</v>
@@ -1158,12 +1158,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1173,17 +1173,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1226,16 +1226,16 @@
         <v>8</v>
       </c>
       <c r="T8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V8" t="n">
         <v>16</v>
       </c>
       <c r="W8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1257,12 +1257,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1272,17 +1272,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1325,16 +1325,16 @@
         <v>9</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="U9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="V9" t="n">
         <v>12</v>
       </c>
       <c r="W9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1356,42 +1356,42 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1424,16 +1424,16 @@
         <v>10</v>
       </c>
       <c r="T10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1523,16 +1523,16 @@
         <v>11</v>
       </c>
       <c r="T11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
         <v>13</v>
       </c>
       <c r="W11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1554,42 +1554,42 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>stimuli/ball/ball_31.jpg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>stimuli/dog/dog_21.jpg</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>stimuli/fish/fish_03.jpg</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_17.jpg</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>stimuli/fish/fish_03.jpg</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_47.jpg</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>ball</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>chair</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>house</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>fish</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>hand</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1622,16 +1622,16 @@
         <v>12</v>
       </c>
       <c r="T12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V12" t="n">
         <v>12</v>
       </c>
       <c r="W12" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1663,17 +1663,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1721,16 +1721,16 @@
         <v>13</v>
       </c>
       <c r="T13" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U13" t="n">
         <v>14</v>
       </c>
       <c r="V13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1829,7 +1829,7 @@
         <v>13</v>
       </c>
       <c r="W14" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1925,10 +1925,10 @@
         <v>13</v>
       </c>
       <c r="V15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1975,12 +1975,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2021,10 +2021,10 @@
         <v>13</v>
       </c>
       <c r="U16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W16" t="n">
         <v>14</v>
@@ -2049,17 +2049,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2117,13 +2117,13 @@
         <v>4</v>
       </c>
       <c r="T17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V17" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W17" t="n">
         <v>16</v>
@@ -2148,19 +2148,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>stimuli/dog/dog_21.jpg</t>
-        </is>
-      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>stimuli/guitar/guitar_19.jpg</t>
@@ -2168,17 +2168,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>jacket</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>dog</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2216,13 +2216,13 @@
         <v>5</v>
       </c>
       <c r="T18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U18" t="n">
+        <v>3</v>
+      </c>
+      <c r="V18" t="n">
         <v>10</v>
-      </c>
-      <c r="V18" t="n">
-        <v>5</v>
       </c>
       <c r="W18" t="n">
         <v>13</v>
@@ -2247,12 +2247,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2262,17 +2262,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2315,16 +2315,16 @@
         <v>6</v>
       </c>
       <c r="T19" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V19" t="n">
         <v>12</v>
       </c>
       <c r="W19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -2346,17 +2346,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2414,13 +2414,13 @@
         <v>7</v>
       </c>
       <c r="T20" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U20" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V20" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="W20" t="n">
         <v>12</v>
@@ -2445,17 +2445,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2465,17 +2465,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2513,13 +2513,13 @@
         <v>8</v>
       </c>
       <c r="T21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V21" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W21" t="n">
         <v>14</v>
@@ -2544,19 +2544,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>stimuli/jacket/jacket_41.jpg</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_17.jpg</t>
-        </is>
-      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>stimuli/pencil/pencil_27.jpg</t>
@@ -2564,17 +2564,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
+          <t>jacket</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t>dog</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>house</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2612,13 +2612,13 @@
         <v>9</v>
       </c>
       <c r="T22" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="U22" t="n">
+        <v>10</v>
+      </c>
+      <c r="V22" t="n">
         <v>5</v>
-      </c>
-      <c r="V22" t="n">
-        <v>9</v>
       </c>
       <c r="W22" t="n">
         <v>16</v>
@@ -2643,42 +2643,42 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2711,16 +2711,16 @@
         <v>10</v>
       </c>
       <c r="T23" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V23" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W23" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -2742,42 +2742,42 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>stimuli/hammer/hammer_10.jpg</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>stimuli/ball/ball_31.jpg</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>stimuli/pencil/pencil_27.jpg</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>stimuli/chair/chair_11.jpg</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>stimuli/flower/flower_32.jpg</t>
-        </is>
-      </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>ball</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>bicycle</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>chair</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>pencil</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>flower</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2810,16 +2810,16 @@
         <v>11</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V24" t="n">
         <v>16</v>
       </c>
       <c r="W24" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -2841,42 +2841,42 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>stimuli/dog/dog_21.jpg</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>stimuli/flower/flower_32.jpg</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>stimuli/ball/ball_31.jpg</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
           <t>house</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>hammer</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>ball</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2909,16 +2909,16 @@
         <v>12</v>
       </c>
       <c r="T25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U25" t="n">
+        <v>5</v>
+      </c>
+      <c r="V25" t="n">
+        <v>6</v>
+      </c>
+      <c r="W25" t="n">
         <v>9</v>
-      </c>
-      <c r="V25" t="n">
-        <v>7</v>
-      </c>
-      <c r="W25" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2950,17 +2950,17 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3008,16 +3008,16 @@
         <v>13</v>
       </c>
       <c r="T26" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U26" t="n">
         <v>14</v>
       </c>
       <c r="V26" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -3049,12 +3049,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3069,12 +3069,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3113,10 +3113,10 @@
         <v>16</v>
       </c>
       <c r="V27" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W27" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -3148,12 +3148,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3168,12 +3168,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3212,10 +3212,10 @@
         <v>13</v>
       </c>
       <c r="V28" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W28" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3262,12 +3262,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3308,10 +3308,10 @@
         <v>13</v>
       </c>
       <c r="U29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V29" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W29" t="n">
         <v>16</v>
@@ -3336,17 +3336,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3356,17 +3356,17 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3404,13 +3404,13 @@
         <v>4</v>
       </c>
       <c r="T30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U30" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V30" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W30" t="n">
         <v>14</v>
@@ -3435,42 +3435,42 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3503,16 +3503,16 @@
         <v>5</v>
       </c>
       <c r="T31" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U31" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V31" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3534,17 +3534,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3554,17 +3554,17 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3602,13 +3602,13 @@
         <v>6</v>
       </c>
       <c r="T32" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U32" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V32" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W32" t="n">
         <v>14</v>
@@ -3633,12 +3633,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3648,17 +3648,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3701,16 +3701,16 @@
         <v>7</v>
       </c>
       <c r="T33" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U33" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V33" t="n">
         <v>13</v>
       </c>
       <c r="W33" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -3732,12 +3732,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3747,17 +3747,17 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3800,16 +3800,16 @@
         <v>8</v>
       </c>
       <c r="T34" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V34" t="n">
         <v>12</v>
       </c>
       <c r="W34" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -3831,42 +3831,42 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3899,16 +3899,16 @@
         <v>9</v>
       </c>
       <c r="T35" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="U35" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="V35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W35" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -3930,17 +3930,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3950,17 +3950,17 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -3998,13 +3998,13 @@
         <v>10</v>
       </c>
       <c r="T36" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U36" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W36" t="n">
         <v>14</v>
@@ -4029,42 +4029,42 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4097,16 +4097,16 @@
         <v>11</v>
       </c>
       <c r="T37" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W37" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38">
@@ -4128,42 +4128,42 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>stimuli/ball/ball_31.jpg</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>stimuli/dog/dog_21.jpg</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>stimuli/pencil/pencil_27.jpg</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_17.jpg</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_47.jpg</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>ball</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
           <t>chair</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>house</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>pencil</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>hand</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4196,16 +4196,16 @@
         <v>12</v>
       </c>
       <c r="T38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U38" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V38" t="n">
         <v>16</v>
       </c>
       <c r="W38" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4242,12 +4242,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4295,7 +4295,7 @@
         <v>13</v>
       </c>
       <c r="T39" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U39" t="n">
         <v>14</v>
@@ -4304,7 +4304,7 @@
         <v>13</v>
       </c>
       <c r="W39" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40">
@@ -4336,12 +4336,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4356,12 +4356,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4400,10 +4400,10 @@
         <v>16</v>
       </c>
       <c r="V40" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W40" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -4499,7 +4499,7 @@
         <v>13</v>
       </c>
       <c r="V41" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="W41" t="n">
         <v>16</v>
@@ -4529,14 +4529,14 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
+          <t>stimuli/flower/flower_32.jpg</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
-        </is>
-      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>stimuli/lamp/lamp_18.jpg</t>
@@ -4549,12 +4549,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
           <t>hammer</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>bicycle</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -4595,10 +4595,10 @@
         <v>13</v>
       </c>
       <c r="U42" t="n">
+        <v>6</v>
+      </c>
+      <c r="V42" t="n">
         <v>7</v>
-      </c>
-      <c r="V42" t="n">
-        <v>2</v>
       </c>
       <c r="W42" t="n">
         <v>14</v>
@@ -4623,42 +4623,42 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4691,16 +4691,16 @@
         <v>4</v>
       </c>
       <c r="T43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U43" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V43" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W43" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -4722,19 +4722,19 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
           <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>stimuli/dog/dog_21.jpg</t>
-        </is>
-      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>stimuli/pencil/pencil_27.jpg</t>
@@ -4742,17 +4742,17 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
           <t>jacket</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>dog</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -4790,13 +4790,13 @@
         <v>5</v>
       </c>
       <c r="T44" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U44" t="n">
+        <v>3</v>
+      </c>
+      <c r="V44" t="n">
         <v>10</v>
-      </c>
-      <c r="V44" t="n">
-        <v>5</v>
       </c>
       <c r="W44" t="n">
         <v>16</v>
@@ -4821,42 +4821,42 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -4889,16 +4889,16 @@
         <v>6</v>
       </c>
       <c r="T45" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U45" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V45" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -4920,42 +4920,42 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -4988,16 +4988,16 @@
         <v>7</v>
       </c>
       <c r="T46" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U46" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V46" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
@@ -5019,42 +5019,42 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5087,16 +5087,16 @@
         <v>8</v>
       </c>
       <c r="T47" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U47" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W47" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -5118,12 +5118,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5138,12 +5138,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -5186,10 +5186,10 @@
         <v>9</v>
       </c>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="U48" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="V48" t="n">
         <v>16</v>
@@ -5217,42 +5217,42 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
+          <t>stimuli/hammer/hammer_10.jpg</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>stimuli/fish/fish_03.jpg</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>stimuli/fish/fish_03.jpg</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>stimuli/flower/flower_32.jpg</t>
-        </is>
-      </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
           <t>bicycle</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>fish</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>flower</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5285,16 +5285,16 @@
         <v>10</v>
       </c>
       <c r="T49" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U49" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V49" t="n">
         <v>12</v>
       </c>
       <c r="W49" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
@@ -5316,17 +5316,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -5336,17 +5336,17 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -5384,13 +5384,13 @@
         <v>11</v>
       </c>
       <c r="T50" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V50" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W50" t="n">
         <v>16</v>
@@ -5415,12 +5415,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5430,17 +5430,17 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5483,16 +5483,16 @@
         <v>12</v>
       </c>
       <c r="T51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U51" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V51" t="n">
         <v>12</v>
       </c>
       <c r="W51" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52">
@@ -5514,42 +5514,42 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>stimuli/dog/dog_21.jpg</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>stimuli/lamp/lamp_18.jpg</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>stimuli/flower/flower_32.jpg</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
           <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>stimuli/lamp/lamp_18.jpg</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>stimuli/ball/ball_31.jpg</t>
-        </is>
-      </c>
       <c r="I52" t="inlineStr">
         <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>lamp</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
           <t>house</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>lamp</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>hammer</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>ball</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -5582,16 +5582,16 @@
         <v>13</v>
       </c>
       <c r="T52" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U52" t="n">
         <v>14</v>
       </c>
       <c r="V52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W52" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -5690,7 +5690,7 @@
         <v>13</v>
       </c>
       <c r="W53" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54">
@@ -5722,12 +5722,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -5786,10 +5786,10 @@
         <v>13</v>
       </c>
       <c r="V54" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W54" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
@@ -5816,12 +5816,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5836,12 +5836,12 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -5882,10 +5882,10 @@
         <v>13</v>
       </c>
       <c r="U55" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V55" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W55" t="n">
         <v>16</v>
@@ -5910,42 +5910,42 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
+          <t>stimuli/jacket/jacket_41.jpg</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
           <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_17.jpg</t>
-        </is>
-      </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
+          <t>jacket</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
           <t>dog</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>house</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -5978,16 +5978,16 @@
         <v>4</v>
       </c>
       <c r="T56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U56" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V56" t="n">
+        <v>10</v>
+      </c>
+      <c r="W56" t="n">
         <v>5</v>
-      </c>
-      <c r="W56" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="57">
@@ -6009,17 +6009,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -6029,17 +6029,17 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -6077,13 +6077,13 @@
         <v>5</v>
       </c>
       <c r="T57" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U57" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V57" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W57" t="n">
         <v>16</v>
@@ -6108,17 +6108,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -6128,17 +6128,17 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -6176,13 +6176,13 @@
         <v>6</v>
       </c>
       <c r="T58" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U58" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V58" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W58" t="n">
         <v>14</v>
@@ -6207,42 +6207,42 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -6275,16 +6275,16 @@
         <v>7</v>
       </c>
       <c r="T59" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U59" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V59" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="W59" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60">
@@ -6306,42 +6306,42 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -6374,16 +6374,16 @@
         <v>8</v>
       </c>
       <c r="T60" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W60" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -6405,19 +6405,19 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
+          <t>stimuli/house/house_17.jpg</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>stimuli/jacket/jacket_41.jpg</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
           <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>stimuli/dog/dog_21.jpg</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>stimuli/chair/chair_11.jpg</t>
-        </is>
-      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>stimuli/guitar/guitar_19.jpg</t>
@@ -6425,17 +6425,17 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
+          <t>house</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>jacket</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
           <t>ball</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>dog</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>chair</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -6473,13 +6473,13 @@
         <v>9</v>
       </c>
       <c r="T61" t="n">
+        <v>9</v>
+      </c>
+      <c r="U61" t="n">
+        <v>10</v>
+      </c>
+      <c r="V61" t="n">
         <v>1</v>
-      </c>
-      <c r="U61" t="n">
-        <v>5</v>
-      </c>
-      <c r="V61" t="n">
-        <v>4</v>
       </c>
       <c r="W61" t="n">
         <v>13</v>
@@ -6504,42 +6504,42 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
+          <t>stimuli/hammer/hammer_10.jpg</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>stimuli/pencil/pencil_27.jpg</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
           <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>stimuli/pencil/pencil_27.jpg</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>stimuli/flower/flower_32.jpg</t>
-        </is>
-      </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
           <t>bicycle</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>pencil</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>flower</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -6572,16 +6572,16 @@
         <v>10</v>
       </c>
       <c r="T62" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U62" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V62" t="n">
         <v>16</v>
       </c>
       <c r="W62" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -6603,12 +6603,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -6618,17 +6618,17 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -6671,16 +6671,16 @@
         <v>11</v>
       </c>
       <c r="T63" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="U63" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V63" t="n">
         <v>12</v>
       </c>
       <c r="W63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64">
@@ -6702,42 +6702,42 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
+          <t>stimuli/ball/ball_31.jpg</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>stimuli/dog/dog_21.jpg</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>stimuli/flower/flower_32.jpg</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
           <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>stimuli/house/house_17.jpg</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_47.jpg</t>
-        </is>
-      </c>
       <c r="I64" t="inlineStr">
         <is>
+          <t>ball</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
           <t>chair</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>house</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>hammer</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>hand</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -6770,16 +6770,16 @@
         <v>12</v>
       </c>
       <c r="T64" t="n">
+        <v>1</v>
+      </c>
+      <c r="U64" t="n">
+        <v>5</v>
+      </c>
+      <c r="V64" t="n">
+        <v>6</v>
+      </c>
+      <c r="W64" t="n">
         <v>4</v>
-      </c>
-      <c r="U64" t="n">
-        <v>9</v>
-      </c>
-      <c r="V64" t="n">
-        <v>7</v>
-      </c>
-      <c r="W64" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -6811,17 +6811,17 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -6831,12 +6831,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -6869,16 +6869,16 @@
         <v>13</v>
       </c>
       <c r="T65" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U65" t="n">
         <v>14</v>
       </c>
       <c r="V65" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W65" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="66">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -6974,7 +6974,7 @@
         <v>16</v>
       </c>
       <c r="V66" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W66" t="n">
         <v>12</v>
@@ -7009,12 +7009,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -7029,12 +7029,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -7073,10 +7073,10 @@
         <v>13</v>
       </c>
       <c r="V67" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="W67" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
@@ -7103,19 +7103,19 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
+          <t>stimuli/bread/bread_21.jpg</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
           <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>stimuli/dog/dog_21.jpg</t>
-        </is>
-      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>guitar</t>
@@ -7123,17 +7123,17 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
           <t>jacket</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>dog</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -7169,13 +7169,13 @@
         <v>13</v>
       </c>
       <c r="U68" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V68" t="n">
+        <v>3</v>
+      </c>
+      <c r="W68" t="n">
         <v>10</v>
-      </c>
-      <c r="W68" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -7197,17 +7197,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -7217,17 +7217,17 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -7265,13 +7265,13 @@
         <v>4</v>
       </c>
       <c r="T69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U69" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V69" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W69" t="n">
         <v>16</v>
@@ -7296,17 +7296,17 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>stimuli/flower/flower_32.jpg</t>
+          <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -7316,17 +7316,17 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>bicycle</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -7364,13 +7364,13 @@
         <v>5</v>
       </c>
       <c r="T70" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U70" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V70" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W70" t="n">
         <v>14</v>
@@ -7395,17 +7395,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>stimuli/bicycle/bicycle_05.jpg</t>
+          <t>stimuli/hammer/hammer_10.jpg</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -7415,17 +7415,17 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>bicycle</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -7463,13 +7463,13 @@
         <v>6</v>
       </c>
       <c r="T71" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="U71" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V71" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="W71" t="n">
         <v>12</v>
@@ -7494,12 +7494,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -7509,17 +7509,17 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -7529,7 +7529,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -7562,16 +7562,16 @@
         <v>7</v>
       </c>
       <c r="T72" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U72" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V72" t="n">
         <v>14</v>
       </c>
       <c r="W72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73">
@@ -7593,12 +7593,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>stimuli/hand/hand_47.jpg</t>
+          <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7608,17 +7608,17 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>hand</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -7661,16 +7661,16 @@
         <v>8</v>
       </c>
       <c r="T73" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U73" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="V73" t="n">
         <v>13</v>
       </c>
       <c r="W73" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
@@ -7692,12 +7692,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -7707,17 +7707,17 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>stimuli/bread/bread_21.jpg</t>
+          <t>stimuli/hand/hand_47.jpg</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>bread</t>
+          <t>hand</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -7760,16 +7760,16 @@
         <v>9</v>
       </c>
       <c r="T74" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="U74" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="V74" t="n">
         <v>14</v>
       </c>
       <c r="W74" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75">
@@ -7791,42 +7791,42 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>stimuli/dog/dog_21.jpg</t>
+          <t>stimuli/jacket/jacket_41.jpg</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
+          <t>stimuli/hammer/hammer_10.jpg</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>stimuli/guitar/guitar_19.jpg</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
           <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>stimuli/guitar/guitar_19.jpg</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>stimuli/flower/flower_32.jpg</t>
-        </is>
-      </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>dog</t>
+          <t>jacket</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>guitar</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
           <t>bicycle</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>guitar</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>flower</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -7859,16 +7859,16 @@
         <v>10</v>
       </c>
       <c r="T75" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U75" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="V75" t="n">
         <v>13</v>
       </c>
       <c r="W75" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
@@ -7890,42 +7890,42 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
+          <t>stimuli/hammer/hammer_10.jpg</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>stimuli/ball/ball_31.jpg</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
           <t>stimuli/bicycle/bicycle_05.jpg</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>stimuli/chair/chair_11.jpg</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>stimuli/flower/flower_32.jpg</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>stimuli/hand/hand_47.jpg</t>
-        </is>
-      </c>
       <c r="I76" t="inlineStr">
         <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>ball</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
           <t>bicycle</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="L76" t="inlineStr">
         <is>
           <t>chair</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>flower</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>hand</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -7958,16 +7958,16 @@
         <v>11</v>
       </c>
       <c r="T76" t="n">
+        <v>7</v>
+      </c>
+      <c r="U76" t="n">
+        <v>1</v>
+      </c>
+      <c r="V76" t="n">
         <v>2</v>
       </c>
-      <c r="U76" t="n">
+      <c r="W76" t="n">
         <v>4</v>
-      </c>
-      <c r="V76" t="n">
-        <v>6</v>
-      </c>
-      <c r="W76" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -7989,12 +7989,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>stimuli/chair/chair_11.jpg</t>
+          <t>stimuli/ball/ball_31.jpg</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -8004,17 +8004,17 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>stimuli/jacket/jacket_41.jpg</t>
+          <t>stimuli/bread/bread_21.jpg</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>ball</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>jacket</t>
+          <t>bread</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -8057,16 +8057,16 @@
         <v>12</v>
       </c>
       <c r="T77" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U77" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V77" t="n">
         <v>12</v>
       </c>
       <c r="W77" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
@@ -8088,7 +8088,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>stimuli/house/house_17.jpg</t>
+          <t>stimuli/dog/dog_21.jpg</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8103,12 +8103,12 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>stimuli/hammer/hammer_10.jpg</t>
+          <t>stimuli/flower/flower_32.jpg</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>house</t>
+          <t>dog</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>flower</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -8156,7 +8156,7 @@
         <v>13</v>
       </c>
       <c r="T78" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U78" t="n">
         <v>14</v>
@@ -8165,7 +8165,7 @@
         <v>16</v>
       </c>
       <c r="W78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>stimuli/ball/ball_31.jpg</t>
+          <t>stimuli/house/house_17.jpg</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>ball</t>
+          <t>house</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -8264,7 +8264,7 @@
         <v>13</v>
       </c>
       <c r="W79" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>